<commit_message>
connection bank xlsx file viewer implementation
</commit_message>
<xml_diff>
--- a/public/Connection Bank Template - DreamShift.xlsx
+++ b/public/Connection Bank Template - DreamShift.xlsx
@@ -55,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -64,10 +64,15 @@
     </font>
     <font>
       <sz val="11.0"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+    </font>
+    <font/>
+    <font>
+      <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
-    <font/>
     <font>
       <color theme="1"/>
       <name val="Arial"/>
@@ -89,8 +94,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9EAD3"/>
-        <bgColor rgb="FFD9EAD3"/>
+        <fgColor rgb="FFB6D7A8"/>
+        <bgColor rgb="FFB6D7A8"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,7 +105,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="8">
     <border/>
     <border>
       <left style="thin">
@@ -122,37 +127,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -202,27 +176,28 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="10" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="11" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="12" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="7" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -445,7 +420,7 @@
     <col customWidth="1" min="4" max="4" width="17.0"/>
     <col customWidth="1" min="5" max="5" width="15.75"/>
     <col customWidth="1" min="6" max="6" width="20.5"/>
-    <col customWidth="1" min="7" max="7" width="21.75"/>
+    <col customWidth="1" min="7" max="12" width="21.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,161 +433,134 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
     </row>
     <row r="2">
-      <c r="A2" s="4"/>
-      <c r="G2" s="5"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="7"/>
     </row>
     <row r="3">
-      <c r="A3" s="4"/>
-      <c r="G3" s="5"/>
+      <c r="A3" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
     </row>
     <row r="4">
-      <c r="A4" s="4"/>
-      <c r="G4" s="5"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
     </row>
     <row r="5">
-      <c r="A5" s="4"/>
-      <c r="G5" s="5"/>
+      <c r="A5" s="10"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
     </row>
     <row r="6">
-      <c r="A6" s="4"/>
-      <c r="G6" s="5"/>
+      <c r="A6" s="10"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
     </row>
     <row r="7">
-      <c r="A7" s="4"/>
-      <c r="G7" s="5"/>
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
     </row>
     <row r="8">
-      <c r="A8" s="4"/>
-      <c r="G8" s="5"/>
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
     </row>
     <row r="9">
-      <c r="A9" s="4"/>
-      <c r="G9" s="5"/>
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
     </row>
     <row r="10">
-      <c r="A10" s="4"/>
-      <c r="G10" s="5"/>
-    </row>
-    <row r="11" ht="17.25" customHeight="1">
-      <c r="A11" s="4"/>
-      <c r="G11" s="5"/>
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
     </row>
     <row r="12">
-      <c r="A12" s="4"/>
-      <c r="G12" s="5"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4"/>
-      <c r="G13" s="5"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4"/>
-      <c r="G14" s="5"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4"/>
-      <c r="G15" s="5"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4"/>
-      <c r="G16" s="5"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4"/>
-      <c r="G17" s="5"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="8"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="11"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>3</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="13"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="13"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="13"/>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="13"/>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="13"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:G18"/>
-    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
extract excel functionlity to reusable component
</commit_message>
<xml_diff>
--- a/public/Connection Bank Template - DreamShift.xlsx
+++ b/public/Connection Bank Template - DreamShift.xlsx
@@ -55,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -64,25 +64,24 @@
     </font>
     <font>
       <sz val="11.0"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
     </font>
-    <font/>
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Docs-Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -105,59 +104,8 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="2">
     <border/>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -176,28 +124,23 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -427,135 +370,120 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="7"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
     </row>
     <row r="7">
-      <c r="A7" s="10"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
     </row>
     <row r="8">
-      <c r="A8" s="10"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
     </row>
     <row r="9">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
     </row>
     <row r="10">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
     </row>
     <row r="11">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
     </row>
     <row r="12">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>